<commit_message>
Week 2: proof patterns up to modus ponens, Kahoot for what they have seen
The lecture reached modus ponens in §2.6.4, so the deck adds a recap of
Def. 2.12-2.15 and an exercise with one direct proof, one indirect proof
and one modus ponens proof. The examples stay clear of last year's
sheet 3 (parity of n^2, a^(2k) - 1, soundness of proof patterns). Lemmas
2.5 and 2.7 are only cited by number, since their formulas are sheet
exercises 2.1.4 and 2.1.1. The recap also mentions lifting (§2.3.5).

The Kahoot is rewritten to cover only propositional logic, quantifiers
and §2.6.1-2.6.4, with the same questions as the private Kahoot copy.
The old one had wrong answers and questions on proof patterns and set
theory the class has not seen yet.
</commit_message>
<xml_diff>
--- a/kahoot/week02.xlsx
+++ b/kahoot/week02.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -82,265 +82,423 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">F |= G means:</t>
+          <t xml:space="preserve">Which of the following is a mathematical statement?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">F -&gt; G is a formula</t>
+          <t xml:space="preserve">71 is a prime number</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">every assignment satisfying F satisfies G</t>
+          <t xml:space="preserve">It might rain today</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">F and G have the same symbols</t>
+          <t xml:space="preserve">A ∧ ¬B</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">G is satisfiable</t>
+          <t xml:space="preserve">x + 1 = 2</t>
         </is>
       </c>
       <c r="F9">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Does A -&gt; B |= not A -&gt; not B hold?</t>
+          <t xml:space="preserve">F ⊨ G means:</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">every truth assignment that makes F true makes G true</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">no, take A=0 and B=1</t>
+          <t xml:space="preserve">F → G is true for at least one truth assignment</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">no, take A=1 and B=1</t>
+          <t xml:space="preserve">G is a tautology</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">only if A is a tautology</t>
+          <t xml:space="preserve">F is satisfiable</t>
         </is>
       </c>
       <c r="F10">
         <v>30</v>
       </c>
       <c r="G10">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Which is always true?</t>
+          <t xml:space="preserve">True or false: B ∧ (A → B) ⊨ A</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">(A-&gt;B) or (B-&gt;A)</t>
+          <t xml:space="preserve">True</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">(A-&gt;B) and (B-&gt;A)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A and not A</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A -&gt; not A</t>
+          <t xml:space="preserve">False</t>
         </is>
       </c>
       <c r="F11">
         <v>30</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">((A-&gt;B) and (B-&gt;C)) and not(A-&gt;C) is:</t>
+          <t xml:space="preserve">Which formula is a tautology?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">a tautology</t>
+          <t xml:space="preserve">A → (A ∨ B)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">satisfiable but not valid</t>
+          <t xml:space="preserve">A → (A ∧ B)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">unsatisfiable</t>
+          <t xml:space="preserve">(A ∨ B) → A</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">satisfiable only if C=1</t>
+          <t xml:space="preserve">A ∧ ¬A</t>
         </is>
       </c>
       <c r="F12">
         <v>30</v>
       </c>
       <c r="G12">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Knights tell the truth, knaves lie. Which question reveals whether the left road is right?</t>
+          <t xml:space="preserve">Which formula is unsatisfiable?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Is A true?</t>
+          <t xml:space="preserve">(A → B) ∧ A ∧ ¬B</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Is A &lt;-&gt; B true?</t>
+          <t xml:space="preserve">(A → B) ∧ ¬A</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Is A and B true?</t>
+          <t xml:space="preserve">A ↔ ¬B</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Is B true?</t>
+          <t xml:space="preserve">A → ¬A</t>
         </is>
       </c>
       <c r="F13">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G13">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">In Z, is 'for all x there is y with xy=1' true?</t>
+          <t xml:space="preserve">For formulas F and G, F → G is a tautology if and only if:</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">F ⊨ G</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">no, x=0 has no inverse</t>
+          <t xml:space="preserve">G ⊨ F</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">only for positive x</t>
+          <t xml:space="preserve">F is a tautology</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">only for prime x</t>
+          <t xml:space="preserve">G is satisfiable</t>
         </is>
       </c>
       <c r="F14">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G14">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">The negation of 'for all x, P(x)' is:</t>
+          <t xml:space="preserve">A ∨ ¬A is a tautology. Why is (B → C) ∨ ¬(B → C) one too?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">for all x, not P(x)</t>
+          <t xml:space="preserve">lifting: replace A by the formula B → C</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">there is x with not P(x)</t>
+          <t xml:space="preserve">de Morgan's rules</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">not there is x with P(x)</t>
+          <t xml:space="preserve">double negation</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">there is x with P(x)</t>
+          <t xml:space="preserve">it is not a tautology</t>
         </is>
       </c>
       <c r="F15">
         <v>30</v>
       </c>
       <c r="G15">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every even number &gt; 2 is a sum of two primes. This statement is:</t>
+          <t xml:space="preserve">True or false: ∀x P(x) ∧ ∀x Q(x) ≡ ∀x (P(x) ∧ Q(x))</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
+          <t xml:space="preserve">True</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">true and proved</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a statement whose truth value is unknown</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">not a statement</t>
+          <t xml:space="preserve">False</t>
         </is>
       </c>
       <c r="F16">
         <v>30</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True or false: ∃x (P(x) ∧ Q(x)) ≡ ∃x P(x) ∧ ∃x Q(x)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+      <c r="F17">
+        <v>30</v>
+      </c>
+      <c r="G17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True or false: ∃y ∀x P(x, y) ⊨ ∀x ∃y P(x, y)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+      <c r="F18">
+        <v>30</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Which formula is equivalent to ¬∀x P(x)?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">∃x ¬P(x)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">∀x ¬P(x)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">¬∃x P(x)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">∃x P(x)</t>
+        </is>
+      </c>
+      <c r="F19">
+        <v>20</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The formula ∃x P(x), with the universe and P not fixed, is:</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a formula, not a mathematical statement</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a true statement</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a false statement</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a tautology</t>
+        </is>
+      </c>
+      <c r="F20">
+        <v>30</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An indirect proof of S ⟹ T:</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assumes T is false and proves S is false</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assumes S is false and proves T is false</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assumes T and proves S</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assumes S and proves T</t>
+        </is>
+      </c>
+      <c r="F21">
+        <v>30</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">To prove S by modus ponens, you find a statement R, prove R, and then prove:</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R ⟹ S</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S ⟹ R</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">¬R ⟹ ¬S</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R ⟹ ¬S</t>
+        </is>
+      </c>
+      <c r="F22">
+        <v>30</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>